<commit_message>
Corrected second weight estimation
</commit_message>
<xml_diff>
--- a/Week_2/Codes/Drone_dataset.xlsx
+++ b/Week_2/Codes/Drone_dataset.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
   <si>
     <t>Name</t>
   </si>
@@ -52,6 +52,9 @@
   </si>
   <si>
     <t xml:space="preserve">Aspect Ratio</t>
+  </si>
+  <si>
+    <t>Empty_weight_ratio</t>
   </si>
   <si>
     <t xml:space="preserve">Yangda Mapird Pro</t>
@@ -631,6 +634,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="14.25"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="25.8515625"/>
+    <col customWidth="1" min="5" max="5" width="12.8515625"/>
+    <col customWidth="1" min="6" max="6" width="11.8515625"/>
+    <col customWidth="1" min="7" max="7" width="12.140625"/>
+    <col customWidth="1" min="8" max="8" width="11.140625"/>
+    <col customWidth="1" min="9" max="9" width="16.00390625"/>
+    <col customWidth="1" min="10" max="10" width="15.7109375"/>
+    <col customWidth="1" min="11" max="11" width="12.8515625"/>
+    <col customWidth="1" min="12" max="12" width="16.00390625"/>
+    <col customWidth="1" min="13" max="13" width="17.140625"/>
+  </cols>
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" t="s">
@@ -669,10 +684,13 @@
       <c r="L1" t="s">
         <v>11</v>
       </c>
+      <c r="M1" t="s">
+        <v>12</v>
+      </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2">
         <v>114.444</v>
@@ -707,13 +725,17 @@
       <c r="L2">
         <v>8.8200000000000003</v>
       </c>
+      <c r="M2">
+        <f>G2/E2</f>
+        <v>0.53333333333333333</v>
+      </c>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3">
         <v>2.23</v>
@@ -745,10 +767,14 @@
       <c r="L3">
         <v>9.0844615379999993</v>
       </c>
+      <c r="M3">
+        <f>G3/E3</f>
+        <v>0.43478260869565216</v>
+      </c>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B4">
         <v>120.23999999999999</v>
@@ -783,10 +809,14 @@
       <c r="L4">
         <v>8.2663043480000002</v>
       </c>
+      <c r="M4">
+        <f>G4/E4</f>
+        <v>0.46860465116279076</v>
+      </c>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B5">
         <v>180</v>
@@ -821,10 +851,14 @@
       <c r="L5">
         <v>12.01923077</v>
       </c>
+      <c r="M5">
+        <f>G5/E5</f>
+        <v>0.45833333333333331</v>
+      </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B6">
         <v>67.896000000000001</v>
@@ -859,10 +893,14 @@
       <c r="L6">
         <v>6</v>
       </c>
+      <c r="M6">
+        <f>G6/E6</f>
+        <v>0.57500000000000007</v>
+      </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B7">
         <v>198</v>
@@ -897,10 +935,14 @@
       <c r="L7">
         <v>12.5</v>
       </c>
+      <c r="M7">
+        <f>G7/E7</f>
+        <v>0.43076923076923074</v>
+      </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B8">
         <v>201.852</v>
@@ -935,10 +977,14 @@
       <c r="L8">
         <v>11.430178570000001</v>
       </c>
+      <c r="M8">
+        <f>G8/E8</f>
+        <v>0.45000000000000001</v>
+      </c>
     </row>
     <row r="9" ht="14.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B9">
         <v>374.39999999999998</v>
@@ -973,10 +1019,14 @@
       <c r="L9">
         <v>12.5</v>
       </c>
+      <c r="M9">
+        <f>G9/E9</f>
+        <v>0.49333333333333335</v>
+      </c>
     </row>
     <row r="10" ht="14.25">
       <c r="A10" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B10">
         <v>100</v>
@@ -1011,10 +1061,14 @@
       <c r="L10">
         <v>5.4627586209999999</v>
       </c>
+      <c r="M10">
+        <f>G10/E10</f>
+        <v>0.46666666666666667</v>
+      </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B11">
         <v>200</v>
@@ -1049,10 +1103,14 @@
       <c r="L11">
         <v>8.480769231</v>
       </c>
+      <c r="M11">
+        <f>G11/E11</f>
+        <v>0.48571428571428571</v>
+      </c>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12">
         <v>10</v>
@@ -1084,10 +1142,14 @@
       <c r="L12">
         <v>12.85714286</v>
       </c>
+      <c r="M12">
+        <f>G12/E12</f>
+        <v>0.59999999999999998</v>
+      </c>
     </row>
     <row r="13" ht="14.25">
       <c r="A13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B13">
         <v>65</v>
@@ -1119,10 +1181,14 @@
       <c r="L13">
         <v>6.3375000000000004</v>
       </c>
+      <c r="M13">
+        <f>G13/E13</f>
+        <v>0.48571428571428571</v>
+      </c>
     </row>
     <row r="14" ht="14.25">
       <c r="A14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B14">
         <v>500</v>
@@ -1154,10 +1220,14 @@
       <c r="L14">
         <v>13.33333333</v>
       </c>
+      <c r="M14">
+        <f>G14/E14</f>
+        <v>0.59999999999999998</v>
+      </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D15">
         <v>35</v>
@@ -1185,6 +1255,10 @@
       </c>
       <c r="L15">
         <v>8.5263157889999999</v>
+      </c>
+      <c r="M15">
+        <f>G15/E15</f>
+        <v>0.47500000000000003</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Added fuselage length code
</commit_message>
<xml_diff>
--- a/Week_2/Codes/Drone_dataset.xlsx
+++ b/Week_2/Codes/Drone_dataset.xlsx
@@ -60,21 +60,36 @@
     <t xml:space="preserve">Yangda Mapird Pro</t>
   </si>
   <si>
+    <t xml:space="preserve">Foxtech Nimbus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">FlyDragon FLY-2100</t>
+  </si>
+  <si>
+    <t>Q200</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yangda Nim- bus Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Black Swift S2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Yangda Mapird Plus</t>
   </si>
   <si>
     <t>-</t>
   </si>
   <si>
-    <t xml:space="preserve">Yangda Nim- bus Pro</t>
-  </si>
-  <si>
     <t xml:space="preserve">Yangda FW- 250</t>
   </si>
   <si>
     <t xml:space="preserve">Avy Aera</t>
   </si>
   <si>
+    <t xml:space="preserve">SkyEye Sierra</t>
+  </si>
+  <si>
     <t xml:space="preserve">Foxtech Baby Shark 260</t>
   </si>
   <si>
@@ -85,21 +100,6 @@
   </si>
   <si>
     <t xml:space="preserve">Wingcopter 178</t>
-  </si>
-  <si>
-    <t xml:space="preserve">FlyDragon FLY-2100</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Black Swift S2</t>
-  </si>
-  <si>
-    <t>Q200</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SkyEye Sierra</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Foxtech Nimbus</t>
   </si>
 </sst>
 </file>
@@ -734,252 +734,240 @@
       <c r="A3" t="s">
         <v>14</v>
       </c>
-      <c r="B3" t="s">
-        <v>15</v>
-      </c>
-      <c r="C3">
-        <v>2.23</v>
-      </c>
       <c r="D3">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="E3">
-        <v>11.5</v>
+        <v>6</v>
       </c>
       <c r="F3">
-        <v>1.5</v>
+        <v>0.80000000000000004</v>
       </c>
       <c r="G3">
-        <v>5</v>
+        <v>2.8500000000000001</v>
       </c>
       <c r="H3">
-        <v>4.7199999999999998</v>
+        <v>2.3500000000000001</v>
       </c>
       <c r="I3">
-        <v>2.4300000000000002</v>
+        <v>1.8</v>
       </c>
       <c r="J3">
-        <v>0.65000000000000002</v>
+        <v>0.38</v>
       </c>
       <c r="K3">
-        <v>1.3999999999999999</v>
+        <v>1.3</v>
       </c>
       <c r="L3">
-        <v>9.0844615379999993</v>
+        <v>8.5263157889999999</v>
       </c>
       <c r="M3">
         <f>G3/E3</f>
-        <v>0.43478260869565216</v>
+        <v>0.47500000000000003</v>
       </c>
     </row>
     <row r="4" ht="14.25">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B4">
-        <v>120.23999999999999</v>
+        <v>200</v>
       </c>
       <c r="C4">
-        <v>1.6699999999999999</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="D4">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="E4">
-        <v>8.5999999999999996</v>
+        <v>7</v>
       </c>
       <c r="F4">
-        <v>2</v>
+        <v>1.2</v>
       </c>
       <c r="G4">
-        <v>4.0300000000000002</v>
+        <v>3.3999999999999999</v>
       </c>
       <c r="H4">
-        <v>2.5600000000000001</v>
+        <v>2.3999999999999999</v>
       </c>
       <c r="I4">
-        <v>1.95</v>
+        <v>2.1000000000000001</v>
       </c>
       <c r="J4">
-        <v>0.46000000000000002</v>
+        <v>0.52000000000000002</v>
       </c>
       <c r="K4">
-        <v>1.3</v>
+        <v>1.2</v>
       </c>
       <c r="L4">
-        <v>8.2663043480000002</v>
+        <v>8.480769231</v>
       </c>
       <c r="M4">
         <f>G4/E4</f>
-        <v>0.46860465116279076</v>
+        <v>0.48571428571428571</v>
       </c>
     </row>
     <row r="5" ht="14.25">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B5">
-        <v>180</v>
+        <v>65</v>
       </c>
       <c r="C5">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="D5">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="E5">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="F5">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="G5">
-        <v>5.5</v>
+        <v>3.3999999999999999</v>
       </c>
       <c r="H5">
-        <v>4.5</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="I5">
-        <v>2.5</v>
+        <v>1.95</v>
       </c>
       <c r="J5">
-        <v>0.52000000000000002</v>
-      </c>
-      <c r="K5">
-        <v>1.3999999999999999</v>
+        <v>0.59999999999999998</v>
       </c>
       <c r="L5">
-        <v>12.01923077</v>
+        <v>6.3375000000000004</v>
       </c>
       <c r="M5">
         <f>G5/E5</f>
-        <v>0.45833333333333331</v>
+        <v>0.48571428571428571</v>
       </c>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B6">
-        <v>67.896000000000001</v>
+        <v>120.23999999999999</v>
       </c>
       <c r="C6">
-        <v>0.92000000000000004</v>
+        <v>1.6699999999999999</v>
       </c>
       <c r="D6">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="E6">
-        <v>12</v>
+        <v>8.5999999999999996</v>
       </c>
       <c r="F6">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="G6">
-        <v>6.9000000000000004</v>
+        <v>4.0300000000000002</v>
       </c>
       <c r="H6">
-        <v>3.6000000000000001</v>
+        <v>2.5600000000000001</v>
       </c>
       <c r="I6">
-        <v>2.3999999999999999</v>
+        <v>1.95</v>
       </c>
       <c r="J6">
-        <v>0.95999999999999996</v>
+        <v>0.46000000000000002</v>
       </c>
       <c r="K6">
         <v>1.3</v>
       </c>
       <c r="L6">
-        <v>6</v>
+        <v>8.2663043480000002</v>
       </c>
       <c r="M6">
         <f>G6/E6</f>
-        <v>0.57500000000000007</v>
+        <v>0.46860465116279076</v>
       </c>
     </row>
     <row r="7" ht="14.25">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B7">
-        <v>198</v>
+        <v>10</v>
       </c>
       <c r="C7">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="D7">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="E7">
-        <v>13</v>
+        <v>9.5</v>
       </c>
       <c r="F7">
-        <v>2.1000000000000001</v>
+        <v>2.2999999999999998</v>
       </c>
       <c r="G7">
-        <v>5.5999999999999996</v>
+        <v>5.7000000000000002</v>
       </c>
       <c r="H7">
-        <v>5.2999999999999998</v>
+        <v>1.5</v>
       </c>
       <c r="I7">
-        <v>2.5</v>
+        <v>3</v>
       </c>
       <c r="J7">
-        <v>0.5</v>
-      </c>
-      <c r="K7">
-        <v>1.4399999999999999</v>
+        <v>0.69999999999999996</v>
       </c>
       <c r="L7">
-        <v>12.5</v>
+        <v>12.85714286</v>
       </c>
       <c r="M7">
         <f>G7/E7</f>
-        <v>0.43076923076923074</v>
+        <v>0.59999999999999998</v>
       </c>
     </row>
     <row r="8" ht="14.25">
       <c r="A8" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" t="s">
         <v>20</v>
       </c>
-      <c r="B8">
-        <v>201.852</v>
-      </c>
       <c r="C8">
-        <v>2.6699999999999999</v>
+        <v>2.23</v>
       </c>
       <c r="D8">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E8">
-        <v>14</v>
+        <v>11.5</v>
       </c>
       <c r="F8">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G8">
-        <v>6.2999999999999998</v>
+        <v>5</v>
       </c>
       <c r="H8">
-        <v>5.7000000000000002</v>
+        <v>4.7199999999999998</v>
       </c>
       <c r="I8">
-        <v>2.5299999999999998</v>
+        <v>2.4300000000000002</v>
       </c>
       <c r="J8">
-        <v>0.56000000000000005</v>
+        <v>0.65000000000000002</v>
       </c>
       <c r="K8">
-        <v>1.21</v>
+        <v>1.3999999999999999</v>
       </c>
       <c r="L8">
-        <v>11.430178570000001</v>
+        <v>9.0844615379999993</v>
       </c>
       <c r="M8">
         <f>G8/E8</f>
-        <v>0.45000000000000001</v>
+        <v>0.43478260869565216</v>
       </c>
     </row>
     <row r="9" ht="14.25">
@@ -987,41 +975,41 @@
         <v>21</v>
       </c>
       <c r="B9">
-        <v>374.39999999999998</v>
+        <v>180</v>
       </c>
       <c r="C9">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D9">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E9">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F9">
-        <v>2.2000000000000002</v>
+        <v>2</v>
       </c>
       <c r="G9">
-        <v>7.4000000000000004</v>
+        <v>5.5</v>
       </c>
       <c r="H9">
-        <v>5.4000000000000004</v>
+        <v>4.5</v>
       </c>
       <c r="I9">
         <v>2.5</v>
       </c>
       <c r="J9">
-        <v>0.5</v>
+        <v>0.52000000000000002</v>
       </c>
       <c r="K9">
-        <v>1.26</v>
+        <v>1.3999999999999999</v>
       </c>
       <c r="L9">
-        <v>12.5</v>
+        <v>12.01923077</v>
       </c>
       <c r="M9">
         <f>G9/E9</f>
-        <v>0.49333333333333335</v>
+        <v>0.45833333333333331</v>
       </c>
     </row>
     <row r="10" ht="14.25">
@@ -1029,41 +1017,41 @@
         <v>22</v>
       </c>
       <c r="B10">
-        <v>100</v>
+        <v>67.896000000000001</v>
       </c>
       <c r="C10">
+        <v>0.92000000000000004</v>
+      </c>
+      <c r="D10">
+        <v>20.5</v>
+      </c>
+      <c r="E10">
+        <v>12</v>
+      </c>
+      <c r="F10">
         <v>1.5</v>
       </c>
-      <c r="D10">
-        <v>42</v>
-      </c>
-      <c r="E10">
-        <v>18</v>
-      </c>
-      <c r="F10">
-        <v>2</v>
-      </c>
       <c r="G10">
-        <v>8.4000000000000004</v>
+        <v>6.9000000000000004</v>
       </c>
       <c r="H10">
-        <v>7.5999999999999996</v>
+        <v>3.6000000000000001</v>
       </c>
       <c r="I10">
-        <v>1.78</v>
+        <v>2.3999999999999999</v>
       </c>
       <c r="J10">
-        <v>0.57999999999999996</v>
+        <v>0.95999999999999996</v>
       </c>
       <c r="K10">
-        <v>1.3200000000000001</v>
+        <v>1.3</v>
       </c>
       <c r="L10">
-        <v>5.4627586209999999</v>
+        <v>6</v>
       </c>
       <c r="M10">
         <f>G10/E10</f>
-        <v>0.46666666666666667</v>
+        <v>0.57500000000000007</v>
       </c>
     </row>
     <row r="11" ht="14.25">
@@ -1071,41 +1059,38 @@
         <v>23</v>
       </c>
       <c r="B11">
-        <v>200</v>
+        <v>500</v>
       </c>
       <c r="C11">
-        <v>2.2999999999999998</v>
+        <v>4.5</v>
       </c>
       <c r="D11">
         <v>18</v>
       </c>
       <c r="E11">
-        <v>7</v>
+        <v>12.5</v>
       </c>
       <c r="F11">
-        <v>1.2</v>
+        <v>5</v>
       </c>
       <c r="G11">
-        <v>3.3999999999999999</v>
-      </c>
-      <c r="H11">
-        <v>2.3999999999999999</v>
+        <v>7.5</v>
       </c>
       <c r="I11">
-        <v>2.1000000000000001</v>
+        <v>2</v>
       </c>
       <c r="J11">
-        <v>0.52000000000000002</v>
+        <v>0.29999999999999999</v>
       </c>
       <c r="K11">
-        <v>1.2</v>
+        <v>1.5</v>
       </c>
       <c r="L11">
-        <v>8.480769231</v>
+        <v>13.33333333</v>
       </c>
       <c r="M11">
         <f>G11/E11</f>
-        <v>0.48571428571428571</v>
+        <v>0.59999999999999998</v>
       </c>
     </row>
     <row r="12" ht="14.25">
@@ -1113,38 +1098,41 @@
         <v>24</v>
       </c>
       <c r="B12">
-        <v>10</v>
+        <v>198</v>
       </c>
       <c r="C12">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="D12">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="E12">
-        <v>9.5</v>
+        <v>13</v>
       </c>
       <c r="F12">
-        <v>2.2999999999999998</v>
+        <v>2.1000000000000001</v>
       </c>
       <c r="G12">
-        <v>5.7000000000000002</v>
+        <v>5.5999999999999996</v>
       </c>
       <c r="H12">
-        <v>1.5</v>
+        <v>5.2999999999999998</v>
       </c>
       <c r="I12">
-        <v>3</v>
+        <v>2.5</v>
       </c>
       <c r="J12">
-        <v>0.69999999999999996</v>
+        <v>0.5</v>
+      </c>
+      <c r="K12">
+        <v>1.4399999999999999</v>
       </c>
       <c r="L12">
-        <v>12.85714286</v>
+        <v>12.5</v>
       </c>
       <c r="M12">
         <f>G12/E12</f>
-        <v>0.59999999999999998</v>
+        <v>0.43076923076923074</v>
       </c>
     </row>
     <row r="13" ht="14.25">
@@ -1152,38 +1140,41 @@
         <v>25</v>
       </c>
       <c r="B13">
-        <v>65</v>
+        <v>201.852</v>
       </c>
       <c r="C13">
-        <v>1.5</v>
+        <v>2.6699999999999999</v>
       </c>
       <c r="D13">
-        <v>12</v>
+        <v>21</v>
       </c>
       <c r="E13">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="F13">
-        <v>2.5</v>
+        <v>2</v>
       </c>
       <c r="G13">
-        <v>3.3999999999999999</v>
+        <v>6.2999999999999998</v>
       </c>
       <c r="H13">
-        <v>1.1000000000000001</v>
+        <v>5.7000000000000002</v>
       </c>
       <c r="I13">
-        <v>1.95</v>
+        <v>2.5299999999999998</v>
       </c>
       <c r="J13">
-        <v>0.59999999999999998</v>
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="K13">
+        <v>1.21</v>
       </c>
       <c r="L13">
-        <v>6.3375000000000004</v>
+        <v>11.430178570000001</v>
       </c>
       <c r="M13">
         <f>G13/E13</f>
-        <v>0.48571428571428571</v>
+        <v>0.45000000000000001</v>
       </c>
     </row>
     <row r="14" ht="14.25">
@@ -1191,77 +1182,89 @@
         <v>26</v>
       </c>
       <c r="B14">
-        <v>500</v>
+        <v>374.39999999999998</v>
       </c>
       <c r="C14">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="D14">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="E14">
+        <v>15</v>
+      </c>
+      <c r="F14">
+        <v>2.2000000000000002</v>
+      </c>
+      <c r="G14">
+        <v>7.4000000000000004</v>
+      </c>
+      <c r="H14">
+        <v>5.4000000000000004</v>
+      </c>
+      <c r="I14">
+        <v>2.5</v>
+      </c>
+      <c r="J14">
+        <v>0.5</v>
+      </c>
+      <c r="K14">
+        <v>1.26</v>
+      </c>
+      <c r="L14">
         <v>12.5</v>
-      </c>
-      <c r="F14">
-        <v>5</v>
-      </c>
-      <c r="G14">
-        <v>7.5</v>
-      </c>
-      <c r="I14">
-        <v>2</v>
-      </c>
-      <c r="J14">
-        <v>0.29999999999999999</v>
-      </c>
-      <c r="K14">
-        <v>1.5</v>
-      </c>
-      <c r="L14">
-        <v>13.33333333</v>
       </c>
       <c r="M14">
         <f>G14/E14</f>
-        <v>0.59999999999999998</v>
+        <v>0.49333333333333335</v>
       </c>
     </row>
     <row r="15" ht="14.25">
       <c r="A15" t="s">
         <v>27</v>
       </c>
+      <c r="B15">
+        <v>100</v>
+      </c>
+      <c r="C15">
+        <v>1.5</v>
+      </c>
       <c r="D15">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="E15">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="F15">
-        <v>0.80000000000000004</v>
+        <v>2</v>
       </c>
       <c r="G15">
-        <v>2.8500000000000001</v>
+        <v>8.4000000000000004</v>
       </c>
       <c r="H15">
-        <v>2.3500000000000001</v>
+        <v>7.5999999999999996</v>
       </c>
       <c r="I15">
-        <v>1.8</v>
+        <v>1.78</v>
       </c>
       <c r="J15">
-        <v>0.38</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="K15">
-        <v>1.3</v>
+        <v>1.3200000000000001</v>
       </c>
       <c r="L15">
-        <v>8.5263157889999999</v>
+        <v>5.4627586209999999</v>
       </c>
       <c r="M15">
         <f>G15/E15</f>
-        <v>0.47500000000000003</v>
+        <v>0.46666666666666667</v>
       </c>
     </row>
   </sheetData>
+  <sortState ref="A2:M15" columnSort="0">
+    <sortCondition sortBy="value" descending="0" ref="E2:E15"/>
+  </sortState>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>
   <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" usePrinterDefaults="1" blackAndWhite="0" draft="0" cellComments="none" useFirstPageNumber="0" errors="displayed" horizontalDpi="600" verticalDpi="0" copies="1"/>

</xml_diff>